<commit_message>
feat: implement receiving reports, simulation, dev reset tools, and export templates
- Added Receiving Report controller, service, and API routes
- Added Simulation & Reset controllers for development testing and demo data management
- Updated Kanban and Purchase Order/Request controllers with enhanced filtering & queries
- Added and updated Excel/XLSB export and import template files
</commit_message>
<xml_diff>
--- a/template_file/BalanceExportTemplate.xlsx
+++ b/template_file/BalanceExportTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project-andum\cmwi\backend-cmw\template_file\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kerjaan\project-toho\Demo\wms-demo\wms-demo-backend\template_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5147A70-E886-4AA0-93B3-177D50024B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7C8094-0E31-4ABA-BF59-753809833681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68B70A97-9B1A-4050-BAC0-10AB1B61C359}"/>
+    <workbookView xWindow="28680" yWindow="-4365" windowWidth="29040" windowHeight="15720" xr2:uid="{68B70A97-9B1A-4050-BAC0-10AB1B61C359}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -231,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -255,7 +255,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -281,45 +280,39 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
+      <xdr:colOff>514351</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>631825</xdr:colOff>
+      <xdr:colOff>819150</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>403225</xdr:rowOff>
+      <xdr:rowOff>382709</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6715E0F-EDF4-4510-AE3F-C4BAC6E4C6D8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6CDFEA6-CA86-E406-F1B6-80340E2D75BB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="123825" y="0"/>
-          <a:ext cx="508000" cy="403225"/>
+          <a:off x="514351" y="57150"/>
+          <a:ext cx="304799" cy="325559"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -332,9 +325,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -372,7 +365,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -478,7 +471,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -620,7 +613,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -648,26 +641,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7"/>
-      <c r="C2" s="11"/>
-      <c r="H2" s="11"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">

</xml_diff>